<commit_message>
feat(demo): state every required EV value in the complete Musterwerk pack
The five documents of demo/series/musterwerk-complete now carry every
required EV attribute with all leaves its schema and template need: a
handover register with document id, title, version, language, VDI 2770
class, file and URI; material, hazardous-substance, spare-part, supplier
and BMS read-out sheets; the clear chemistry name, manufacturer address,
cell resistance and original power capability.

completePack.test.ts applies 22 hand decisions on top of the automatic
chain, checks that every leaf is written in its named document, and
proves the result validates and emits valid at 100 % mandatory
completeness. The automatic chain alone stays invalid at 61.7 % with 39
attributes mapped. Base fixtures and musterwerk-12 are byte-identical.
</commit_message>
<xml_diff>
--- a/demo/series/musterwerk-complete/stueckliste.xlsx
+++ b/demo/series/musterwerk-complete/stueckliste.xlsx
@@ -5,12 +5,17 @@
     <sheet name="Stammdaten" sheetId="1" r:id="rId1"/>
     <sheet name="Stückliste" sheetId="2" r:id="rId2"/>
     <sheet name="Leistung" sheetId="3" r:id="rId3"/>
+    <sheet name="Materialdeklaration" sheetId="4" r:id="rId4"/>
+    <sheet name="Gefahrstoffe" sheetId="5" r:id="rId5"/>
+    <sheet name="Ersatzteile" sheetId="6" r:id="rId6"/>
+    <sheet name="Bezugsquellen" sheetId="7" r:id="rId7"/>
+    <sheet name="BMS-Auslesung" sheetId="8" r:id="rId8"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="58">
   <si>
     <t>Batteriepass-ID</t>
   </si>
@@ -81,6 +86,9 @@
     <t>Innenwiderstand Pack</t>
   </si>
   <si>
+    <t>Innenwiderstand Zelle</t>
+  </si>
+  <si>
     <t>Anfänglicher Round-Trip-Wirkungsgrad</t>
   </si>
   <si>
@@ -97,6 +105,90 @@
   </si>
   <si>
     <t>Erschöpfungsschwelle</t>
+  </si>
+  <si>
+    <t>Komponente</t>
+  </si>
+  <si>
+    <t>Kritischer Rohstoff</t>
+  </si>
+  <si>
+    <t>Lithium</t>
+  </si>
+  <si>
+    <t>Cobalt</t>
+  </si>
+  <si>
+    <t>Natural graphite</t>
+  </si>
+  <si>
+    <t>Copper</t>
+  </si>
+  <si>
+    <t>Lithium hexafluorophosphate</t>
+  </si>
+  <si>
+    <t>Stoff</t>
+  </si>
+  <si>
+    <t>Gefahrenklasse</t>
+  </si>
+  <si>
+    <t>Konzentration [%]</t>
+  </si>
+  <si>
+    <t>Gefahrenhinweise</t>
+  </si>
+  <si>
+    <t>Teilenummer</t>
+  </si>
+  <si>
+    <t>Bezugsquelle</t>
+  </si>
+  <si>
+    <t>Battery management system</t>
+  </si>
+  <si>
+    <t>Battery module</t>
+  </si>
+  <si>
+    <t>Cooling plate</t>
+  </si>
+  <si>
+    <t>Lieferant</t>
+  </si>
+  <si>
+    <t>Straße</t>
+  </si>
+  <si>
+    <t>PLZ</t>
+  </si>
+  <si>
+    <t>Land</t>
+  </si>
+  <si>
+    <t>E-Mail</t>
+  </si>
+  <si>
+    <t>Website</t>
+  </si>
+  <si>
+    <t>Musterwerk Ersatzteile GmbH</t>
+  </si>
+  <si>
+    <t>Zeitstempel</t>
+  </si>
+  <si>
+    <t>State of Certified Energy (SOCE)</t>
+  </si>
+  <si>
+    <t>Ladezustand (SoC)</t>
+  </si>
+  <si>
+    <t>Anzahl Vollzyklen</t>
+  </si>
+  <si>
+    <t>Batterietemperatur</t>
   </si>
 </sst>
 </file>
@@ -226,7 +318,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>siehe Materialdeklaration</t>
         </is>
       </c>
       <c r="C2">
@@ -343,11 +435,11 @@
         <v>23</v>
       </c>
       <c r="B6">
-        <v>96</v>
+        <v>0.0012</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>Ohm</t>
         </is>
       </c>
     </row>
@@ -356,7 +448,7 @@
         <v>24</v>
       </c>
       <c r="B7">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -369,11 +461,11 @@
         <v>25</v>
       </c>
       <c r="B8">
-        <v>110</v>
+        <v>93</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>kW</t>
+          <t>%</t>
         </is>
       </c>
     </row>
@@ -382,11 +474,11 @@
         <v>26</v>
       </c>
       <c r="B9">
-        <v>12</v>
+        <v>110</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Jahre</t>
+          <t>kW</t>
         </is>
       </c>
     </row>
@@ -395,11 +487,11 @@
         <v>27</v>
       </c>
       <c r="B10">
-        <v>0.5</v>
+        <v>12</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>Jahre</t>
         </is>
       </c>
     </row>
@@ -408,11 +500,435 @@
         <v>28</v>
       </c>
       <c r="B11">
+        <v>0.5</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>29</v>
+      </c>
+      <c r="B12">
         <v>70</v>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>%</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>7439-93-2</t>
+        </is>
+      </c>
+      <c r="C2">
+        <v>6.4</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Cathode</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>7440-48-4</t>
+        </is>
+      </c>
+      <c r="C3">
+        <v>4.1</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Cathode</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>7782-42-5</t>
+        </is>
+      </c>
+      <c r="C4">
+        <v>38</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Anode</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>35</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>7440-50-8</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Anode</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>21324-40-3</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Electrolyte</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>21324-40-3</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>AcuteToxicity</t>
+        </is>
+      </c>
+      <c r="D2">
+        <v>1.2</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Electrolyte</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>H301 Toxic if swallowed; H314 Causes severe skin burns and eye damage</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>MW-BMS-7</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Musterwerk Batteriesysteme GmbH</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>MW-MOD-48-A</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Musterwerk Ersatzteile GmbH</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>45</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>MW-CP-12</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Musterwerk Ersatzteile GmbH</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E1" t="s">
+        <v>50</v>
+      </c>
+      <c r="F1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Werkstrasse 2</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>28199</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>ersatzteile@musterwerk.example</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>https://ersatzteile.musterwerk.example</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B2">
+        <v>99.5</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-08-31T06:00:00Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B3">
+        <v>70</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2026-08-31T06:00:00Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>56</v>
+      </c>
+      <c r="B4">
+        <v>12</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Zyklen</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2026-08-30T18:30:00Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>57</v>
+      </c>
+      <c r="B5">
+        <v>23.5</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>°C</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2026-08-31T06:00:00Z</t>
         </is>
       </c>
     </row>

</xml_diff>